<commit_message>
Add 9 blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 24
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-home.report.xlsx
+++ b/tools/importer/reports/import-home.report.xlsx
@@ -52,7 +52,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-10-23T09:35:39.458Z</t>
+    <t>2026-10-23T09:45:41.262Z</t>
   </si>
   <si>
     <t>BANDIT BUNNY</t>
@@ -73,7 +73,7 @@
     <t>blogs</t>
   </si>
   <si>
-    <t>2026-10-23T09:25:18.195Z</t>
+    <t>2026-10-23T09:36:08.910Z</t>
   </si>
   <si>
     <t>Neuigkeiten – BANDIT BUNNY</t>
@@ -94,7 +94,7 @@
     <t>pages</t>
   </si>
   <si>
-    <t>2026-10-23T09:22:47.271Z</t>
+    <t>2026-10-23T09:35:50.404Z</t>
   </si>
   <si>
     <t>Kontakt – BANDIT BUNNY</t>
@@ -109,7 +109,7 @@
     <t>pages/handleranfrage</t>
   </si>
   <si>
-    <t>2026-10-23T09:22:55.575Z</t>
+    <t>2026-10-23T09:35:58.498Z</t>
   </si>
   <si>
     <t>Händleranfrage – BANDIT BUNNY</t>

</xml_diff>